<commit_message>
Document the polygon worksheet in the input template guide
Add a "Worksheet: polygon" section (and structure-table row) describing
the polygon sheet as an alternative to profile lines for defining slope
geometry as closed material zones, with a worksheet screenshot.

Also update the edited Lost Lake polygon example file.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/poly_test/xslope_lost_lake_poly.xlsx
+++ b/poly_test/xslope_lost_lake_poly.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/poly_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3293A3-B1F8-4840-BCCF-D44260C5241D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25040" yWindow="2500" windowWidth="42700" windowHeight="22800" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="25040" yWindow="2500" windowWidth="42700" windowHeight="22800" activeTab="4" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <definedName name="solution2">mat!#REF!</definedName>
     <definedName name="version">main!$D$5</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="189">
   <si>
     <t>X</t>
   </si>
@@ -752,6 +752,30 @@
   </si>
   <si>
     <t>Fixity</t>
+  </si>
+  <si>
+    <t>Rip Rap</t>
+  </si>
+  <si>
+    <t>Shell</t>
+  </si>
+  <si>
+    <t>Clay Core</t>
+  </si>
+  <si>
+    <t>Drain</t>
+  </si>
+  <si>
+    <t>Filter</t>
+  </si>
+  <si>
+    <t>Glacial Till</t>
+  </si>
+  <si>
+    <t>Grouted Bedrock</t>
+  </si>
+  <si>
+    <t>Bedrock</t>
   </si>
 </sst>
 </file>
@@ -1209,13 +1233,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5942,6 +5966,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>316</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>324</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>475</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -5951,6 +5990,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>230</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>198</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -6011,6 +6065,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>225</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6020,6 +6083,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>225</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -6770,6 +6842,24 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>225</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>150</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6779,6 +6869,24 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>225</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>230</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>200</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -6839,6 +6947,27 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>240</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6848,6 +6977,27 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>230</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>230</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>230</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -6908,6 +7058,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>316</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>313</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>260</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6917,6 +7082,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>230</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>230</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -6977,6 +7157,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>153</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6986,6 +7178,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>200</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7049,6 +7253,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>215</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>210</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7058,6 +7286,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>200</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7121,6 +7373,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>313</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>260</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7130,6 +7394,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>229</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7193,6 +7469,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>313</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>316</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>255</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7202,6 +7502,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>229</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7265,6 +7589,39 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>324</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>253</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>245</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>240</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7274,6 +7631,39 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>190</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7337,6 +7727,27 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>215</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7346,6 +7757,27 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>200</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7409,6 +7841,24 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>253</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>324</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>475</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>475</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7418,6 +7868,24 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>195</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7478,6 +7946,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>220</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7487,6 +7970,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>190</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -7547,6 +8045,42 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>215</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>245</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>475</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>475</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7556,6 +8090,42 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>195</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -11494,7 +12064,7 @@
         <v>95</v>
       </c>
       <c r="F3" s="38">
-        <v>225.0</v>
+        <v>225</v>
       </c>
       <c r="H3" s="37" t="s">
         <v>95</v>
@@ -11553,16 +12123,16 @@
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="C5" s="3">
-        <v>230.0</v>
+        <v>230</v>
       </c>
       <c r="E5" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -11575,16 +12145,16 @@
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
-        <v>316.0</v>
+        <v>316</v>
       </c>
       <c r="C6" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="E6" s="3">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="F6" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -11597,16 +12167,16 @@
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B7" s="3">
-        <v>320.0</v>
+        <v>320</v>
       </c>
       <c r="C7" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="E7" s="3">
-        <v>225.0</v>
+        <v>225</v>
       </c>
       <c r="F7" s="3">
-        <v>225.0</v>
+        <v>225</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -11619,10 +12189,10 @@
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B8" s="3">
-        <v>324.0</v>
+        <v>324</v>
       </c>
       <c r="C8" s="3">
-        <v>198.0</v>
+        <v>198</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -11637,10 +12207,10 @@
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B9" s="3">
-        <v>475.0</v>
+        <v>475</v>
       </c>
       <c r="C9" s="3">
-        <v>198.0</v>
+        <v>198</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -12464,10 +13034,8 @@
       <c r="A9" s="3">
         <v>1</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Rip Rap</t>
-        </is>
+      <c r="B9" s="3" t="s">
+        <v>181</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -12494,7 +13062,7 @@
         <v>0</v>
       </c>
       <c r="U9" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V9" s="3">
         <v>-1</v>
@@ -12506,10 +13074,8 @@
       <c r="A10" s="3">
         <v>2</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Shell</t>
-        </is>
+      <c r="B10" s="3" t="s">
+        <v>182</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -12536,7 +13102,7 @@
         <v>0</v>
       </c>
       <c r="U10" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V10" s="3">
         <v>-1</v>
@@ -12548,10 +13114,8 @@
       <c r="A11" s="3">
         <v>3</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Clay Core</t>
-        </is>
+      <c r="B11" s="3" t="s">
+        <v>183</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -12578,7 +13142,7 @@
         <v>0</v>
       </c>
       <c r="U11" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V11" s="3">
         <v>-1</v>
@@ -12590,10 +13154,8 @@
       <c r="A12" s="3">
         <v>4</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Drain</t>
-        </is>
+      <c r="B12" s="3" t="s">
+        <v>184</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -12620,7 +13182,7 @@
         <v>0</v>
       </c>
       <c r="U12" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V12" s="3">
         <v>-1</v>
@@ -12632,10 +13194,8 @@
       <c r="A13" s="3">
         <v>5</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Filter</t>
-        </is>
+      <c r="B13" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -12662,7 +13222,7 @@
         <v>0</v>
       </c>
       <c r="U13" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V13" s="3">
         <v>-1</v>
@@ -12674,10 +13234,8 @@
       <c r="A14" s="3">
         <v>6</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Glacial Till</t>
-        </is>
+      <c r="B14" s="3" t="s">
+        <v>186</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -12704,7 +13262,7 @@
         <v>0</v>
       </c>
       <c r="U14" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V14" s="3">
         <v>-1</v>
@@ -12716,10 +13274,8 @@
       <c r="A15" s="3">
         <v>7</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Grouted Bedrock</t>
-        </is>
+      <c r="B15" s="3" t="s">
+        <v>187</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -12746,7 +13302,7 @@
         <v>0</v>
       </c>
       <c r="U15" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V15" s="3">
         <v>-1</v>
@@ -12758,10 +13314,8 @@
       <c r="A16" s="3">
         <v>8</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Bedrock</t>
-        </is>
+      <c r="B16" s="3" t="s">
+        <v>188</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -12788,7 +13342,7 @@
         <v>0</v>
       </c>
       <c r="U16" s="3">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="V16" s="3">
         <v>-1</v>
@@ -13354,74 +13908,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="D4" s="50" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="G4" s="50" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="J4" s="50" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="50"/>
-      <c r="M4" s="50" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="50"/>
-      <c r="P4" s="50" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="50"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="50" t="s">
+      <c r="S4" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="50"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="50" t="s">
+      <c r="V4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="50"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="50" t="s">
+      <c r="Y4" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="50"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="50" t="s">
+      <c r="AB4" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="50"/>
-      <c r="AE4" s="50" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="50"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="50" t="s">
+      <c r="AH4" s="52" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="50"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="50" t="s">
+      <c r="AK4" s="52" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="50" t="s">
+      <c r="AN4" s="52" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="50"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="50" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="50"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -13524,89 +14078,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="51" t="str">
+      <c r="A6" s="50" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="B6" s="52"/>
-      <c r="D6" s="51" t="str">
+        <v>Rip Rap</v>
+      </c>
+      <c r="B6" s="51"/>
+      <c r="D6" s="50" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="E6" s="52"/>
-      <c r="G6" s="51" t="str">
+        <v>Shell</v>
+      </c>
+      <c r="E6" s="51"/>
+      <c r="G6" s="50" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="H6" s="52"/>
-      <c r="J6" s="51" t="str">
+        <v>Clay Core</v>
+      </c>
+      <c r="H6" s="51"/>
+      <c r="J6" s="50" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="K6" s="52"/>
-      <c r="M6" s="51" t="str">
+        <v>Drain</v>
+      </c>
+      <c r="K6" s="51"/>
+      <c r="M6" s="50" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="N6" s="52"/>
-      <c r="P6" s="51" t="str">
+        <v>Filter</v>
+      </c>
+      <c r="N6" s="51"/>
+      <c r="P6" s="50" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="Q6" s="52"/>
+        <v>Glacial Till</v>
+      </c>
+      <c r="Q6" s="51"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="51" t="str">
+      <c r="S6" s="50" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="T6" s="52"/>
+        <v>Grouted Bedrock</v>
+      </c>
+      <c r="T6" s="51"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="51" t="str">
+      <c r="V6" s="50" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="W6" s="52"/>
+        <v>Bedrock</v>
+      </c>
+      <c r="W6" s="51"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="51" t="str">
+      <c r="Y6" s="50" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="52"/>
+      <c r="Z6" s="51"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="51" t="str">
+      <c r="AB6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="52"/>
-      <c r="AE6" s="51" t="str">
+      <c r="AC6" s="51"/>
+      <c r="AE6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="52"/>
+      <c r="AF6" s="51"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="51" t="str">
+      <c r="AH6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="52"/>
+      <c r="AI6" s="51"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="51" t="str">
+      <c r="AK6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="52"/>
+      <c r="AL6" s="51"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="51" t="str">
+      <c r="AN6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="52"/>
+      <c r="AO6" s="51"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="51" t="str">
+      <c r="AQ6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="52"/>
+      <c r="AR6" s="51"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -14510,36 +15064,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14577,74 +15131,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="52" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="D4" s="50" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="G4" s="50" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="J4" s="50" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="50"/>
-      <c r="M4" s="50" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="50"/>
-      <c r="P4" s="50" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="50"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="50" t="s">
+      <c r="S4" s="52" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="50"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="50" t="s">
+      <c r="V4" s="52" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="50"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="50" t="s">
+      <c r="Y4" s="52" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="50"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="50" t="s">
+      <c r="AB4" s="52" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="50"/>
-      <c r="AE4" s="50" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="50"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="50" t="s">
+      <c r="AH4" s="52" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="50"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="50" t="s">
+      <c r="AK4" s="52" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="50" t="s">
+      <c r="AN4" s="52" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="50"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="50" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="50"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -14749,67 +15303,67 @@
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="53" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Rip Rap</v>
       </c>
       <c r="B6" s="54"/>
       <c r="D6" s="53" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Shell</v>
       </c>
       <c r="E6" s="54"/>
       <c r="G6" s="53" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Rip Rap</v>
       </c>
       <c r="H6" s="54"/>
       <c r="J6" s="53" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Shell</v>
       </c>
       <c r="K6" s="54"/>
       <c r="M6" s="53" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Clay Core</v>
       </c>
       <c r="N6" s="54"/>
       <c r="P6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Shell</v>
       </c>
       <c r="Q6" s="54"/>
       <c r="R6" s="1"/>
       <c r="S6" s="53" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Drain</v>
       </c>
       <c r="T6" s="54"/>
       <c r="U6" s="1"/>
       <c r="V6" s="53" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Filter</v>
       </c>
       <c r="W6" s="54"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Glacial Till</v>
       </c>
       <c r="Z6" s="54"/>
       <c r="AA6" s="1"/>
       <c r="AB6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Glacial Till</v>
       </c>
       <c r="AC6" s="54"/>
       <c r="AE6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Grouted Bedrock</v>
       </c>
       <c r="AF6" s="54"/>
       <c r="AG6" s="1"/>
       <c r="AH6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Bedrock</v>
       </c>
       <c r="AI6" s="54"/>
       <c r="AJ6" s="1"/>
@@ -14933,81 +15487,81 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="B8" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="D8" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="E8" s="3">
-        <v>230.0</v>
+        <v>230</v>
       </c>
       <c r="G8" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="H8" s="3">
-        <v>230.0</v>
+        <v>230</v>
       </c>
       <c r="J8" s="3">
-        <v>153.0</v>
+        <v>153</v>
       </c>
       <c r="K8" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="M8" s="3">
-        <v>210.0</v>
+        <v>210</v>
       </c>
       <c r="N8" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="P8" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="Q8" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="R8" s="1"/>
       <c r="S8" s="3">
-        <v>255.0</v>
+        <v>255</v>
       </c>
       <c r="T8" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="U8" s="1"/>
       <c r="V8" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="W8" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="X8" s="1"/>
       <c r="Y8" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="AA8" s="1"/>
       <c r="AB8" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="AC8" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AE8" s="3">
-        <v>220.0</v>
+        <v>220</v>
       </c>
       <c r="AF8" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="AG8" s="1"/>
       <c r="AH8" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AI8" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="3"/>
@@ -15021,81 +15575,81 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>225.0</v>
+        <v>225</v>
       </c>
       <c r="B9" s="3">
-        <v>225.0</v>
+        <v>225</v>
       </c>
       <c r="D9" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="E9" s="3">
-        <v>230.0</v>
+        <v>230</v>
       </c>
       <c r="G9" s="3">
-        <v>316.0</v>
+        <v>316</v>
       </c>
       <c r="H9" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="J9" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="K9" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="M9" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="N9" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="P9" s="3">
-        <v>313.0</v>
+        <v>313</v>
       </c>
       <c r="Q9" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="R9" s="1"/>
       <c r="S9" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="T9" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="U9" s="1"/>
       <c r="V9" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="W9" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="X9" s="1"/>
       <c r="Y9" s="3">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="Z9" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="AA9" s="1"/>
       <c r="AB9" s="3">
-        <v>253.0</v>
+        <v>253</v>
       </c>
       <c r="AC9" s="3">
-        <v>198.0</v>
+        <v>198</v>
       </c>
       <c r="AE9" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="AF9" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="AG9" s="1"/>
       <c r="AH9" s="3">
-        <v>215.0</v>
+        <v>215</v>
       </c>
       <c r="AI9" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AJ9" s="1"/>
       <c r="AK9" s="3"/>
@@ -15109,81 +15663,81 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="B10" s="3">
-        <v>230.0</v>
+        <v>230</v>
       </c>
       <c r="D10" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="E10" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="G10" s="3">
-        <v>313.0</v>
+        <v>313</v>
       </c>
       <c r="H10" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="J10" s="3">
-        <v>210.0</v>
+        <v>210</v>
       </c>
       <c r="K10" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="M10" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="N10" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="P10" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="Q10" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="R10" s="1"/>
       <c r="S10" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="T10" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="U10" s="1"/>
       <c r="V10" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="W10" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="X10" s="1"/>
       <c r="Y10" s="3">
-        <v>153.0</v>
+        <v>153</v>
       </c>
       <c r="Z10" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="AA10" s="1"/>
       <c r="AB10" s="3">
-        <v>324.0</v>
+        <v>324</v>
       </c>
       <c r="AC10" s="3">
-        <v>198.0</v>
+        <v>198</v>
       </c>
       <c r="AE10" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="AF10" s="3">
-        <v>140.0</v>
+        <v>140</v>
       </c>
       <c r="AG10" s="1"/>
       <c r="AH10" s="3">
-        <v>220.0</v>
+        <v>220</v>
       </c>
       <c r="AI10" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="AJ10" s="1"/>
       <c r="AK10" s="3"/>
@@ -15197,81 +15751,81 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="B11" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="D11" s="3">
-        <v>255.0</v>
+        <v>255</v>
       </c>
       <c r="E11" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="G11" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="H11" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="J11" s="3">
-        <v>153.0</v>
+        <v>153</v>
       </c>
       <c r="K11" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="M11" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="N11" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="P11" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="Q11" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="R11" s="1"/>
       <c r="S11" s="3">
-        <v>313.0</v>
+        <v>313</v>
       </c>
       <c r="T11" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="U11" s="1"/>
       <c r="V11" s="3">
-        <v>255.0</v>
+        <v>255</v>
       </c>
       <c r="W11" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="X11" s="1"/>
       <c r="Y11" s="3">
-        <v>210.0</v>
+        <v>210</v>
       </c>
       <c r="Z11" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="AA11" s="1"/>
       <c r="AB11" s="3">
-        <v>475.0</v>
+        <v>475</v>
       </c>
       <c r="AC11" s="3">
-        <v>198.0</v>
+        <v>198</v>
       </c>
       <c r="AE11" s="3">
-        <v>220.0</v>
+        <v>220</v>
       </c>
       <c r="AF11" s="3">
-        <v>140.0</v>
+        <v>140</v>
       </c>
       <c r="AG11" s="1"/>
       <c r="AH11" s="3">
-        <v>220.0</v>
+        <v>220</v>
       </c>
       <c r="AI11" s="3">
-        <v>140.0</v>
+        <v>140</v>
       </c>
       <c r="AJ11" s="1"/>
       <c r="AK11" s="3"/>
@@ -15285,73 +15839,73 @@
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>153.0</v>
+        <v>153</v>
       </c>
       <c r="B12" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="D12" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="E12" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="G12" s="3">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="H12" s="3">
-        <v>230.0</v>
+        <v>230</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
       <c r="M12" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="N12" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
       <c r="R12" s="1"/>
       <c r="S12" s="3">
-        <v>316.0</v>
+        <v>316</v>
       </c>
       <c r="T12" s="3">
-        <v>202.0</v>
+        <v>202</v>
       </c>
       <c r="U12" s="1"/>
       <c r="V12" s="3">
-        <v>255.0</v>
+        <v>255</v>
       </c>
       <c r="W12" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="X12" s="1"/>
       <c r="Y12" s="3">
-        <v>215.0</v>
+        <v>215</v>
       </c>
       <c r="Z12" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AA12" s="1"/>
       <c r="AB12" s="3">
-        <v>475.0</v>
+        <v>475</v>
       </c>
       <c r="AC12" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AE12" s="3">
-        <v>220.0</v>
+        <v>220</v>
       </c>
       <c r="AF12" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="AG12" s="1"/>
       <c r="AH12" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="AI12" s="3">
-        <v>140.0</v>
+        <v>140</v>
       </c>
       <c r="AJ12" s="1"/>
       <c r="AK12" s="3"/>
@@ -15365,65 +15919,65 @@
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="B13" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="D13" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="E13" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="M13" s="3">
-        <v>220.0</v>
+        <v>220</v>
       </c>
       <c r="N13" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
       <c r="R13" s="1"/>
       <c r="S13" s="3">
-        <v>320.0</v>
+        <v>320</v>
       </c>
       <c r="T13" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="U13" s="1"/>
       <c r="V13" s="3">
-        <v>320.0</v>
+        <v>320</v>
       </c>
       <c r="W13" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="X13" s="1"/>
       <c r="Y13" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AA13" s="1"/>
       <c r="AB13" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="AC13" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AE13" s="3"/>
       <c r="AF13" s="3"/>
       <c r="AG13" s="1"/>
       <c r="AH13" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="AI13" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="AJ13" s="1"/>
       <c r="AK13" s="3"/>
@@ -15439,43 +15993,43 @@
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="E14" s="3">
-        <v>230.0</v>
+        <v>230</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="M14" s="3">
-        <v>215.0</v>
+        <v>215</v>
       </c>
       <c r="N14" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
       <c r="R14" s="1"/>
       <c r="S14" s="3">
-        <v>255.0</v>
+        <v>255</v>
       </c>
       <c r="T14" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="U14" s="1"/>
       <c r="V14" s="3">
-        <v>324.0</v>
+        <v>324</v>
       </c>
       <c r="W14" s="3">
-        <v>198.0</v>
+        <v>198</v>
       </c>
       <c r="X14" s="1"/>
       <c r="Y14" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z14" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="AA14" s="1"/>
       <c r="AB14" s="3"/>
@@ -15484,10 +16038,10 @@
       <c r="AF14" s="3"/>
       <c r="AG14" s="1"/>
       <c r="AH14" s="3">
-        <v>245.0</v>
+        <v>245</v>
       </c>
       <c r="AI14" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="AJ14" s="1"/>
       <c r="AK14" s="3"/>
@@ -15509,26 +16063,26 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="M15" s="3">
-        <v>210.0</v>
+        <v>210</v>
       </c>
       <c r="N15" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
       <c r="R15" s="1"/>
       <c r="S15" s="3">
-        <v>255.0</v>
+        <v>255</v>
       </c>
       <c r="T15" s="3">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="U15" s="1"/>
       <c r="V15" s="3">
-        <v>253.0</v>
+        <v>253</v>
       </c>
       <c r="W15" s="3">
-        <v>198.0</v>
+        <v>198</v>
       </c>
       <c r="X15" s="1"/>
       <c r="Y15" s="3"/>
@@ -15540,10 +16094,10 @@
       <c r="AF15" s="3"/>
       <c r="AG15" s="1"/>
       <c r="AH15" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="AI15" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AJ15" s="1"/>
       <c r="AK15" s="3"/>
@@ -15573,10 +16127,10 @@
       <c r="T16" s="3"/>
       <c r="U16" s="1"/>
       <c r="V16" s="3">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="W16" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="X16" s="1"/>
       <c r="Y16" s="3"/>
@@ -15588,10 +16142,10 @@
       <c r="AF16" s="3"/>
       <c r="AG16" s="1"/>
       <c r="AH16" s="3">
-        <v>475.0</v>
+        <v>475</v>
       </c>
       <c r="AI16" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AJ16" s="1"/>
       <c r="AK16" s="3"/>
@@ -15621,10 +16175,10 @@
       <c r="T17" s="3"/>
       <c r="U17" s="1"/>
       <c r="V17" s="3">
-        <v>245.0</v>
+        <v>245</v>
       </c>
       <c r="W17" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="X17" s="1"/>
       <c r="Y17" s="3"/>
@@ -15636,10 +16190,10 @@
       <c r="AF17" s="3"/>
       <c r="AG17" s="1"/>
       <c r="AH17" s="3">
-        <v>475.0</v>
+        <v>475</v>
       </c>
       <c r="AI17" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AJ17" s="1"/>
       <c r="AK17" s="3"/>
@@ -15669,10 +16223,10 @@
       <c r="T18" s="3"/>
       <c r="U18" s="1"/>
       <c r="V18" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="W18" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="X18" s="1"/>
       <c r="Y18" s="3"/>
@@ -15684,10 +16238,10 @@
       <c r="AF18" s="3"/>
       <c r="AG18" s="1"/>
       <c r="AH18" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AI18" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AJ18" s="1"/>
       <c r="AK18" s="3"/>
@@ -15728,10 +16282,10 @@
       <c r="AF19" s="3"/>
       <c r="AG19" s="1"/>
       <c r="AH19" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AI19" s="3">
-        <v>195.0</v>
+        <v>195</v>
       </c>
       <c r="AJ19" s="1"/>
       <c r="AK19" s="3"/>
@@ -16065,14 +16619,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -16089,12 +16641,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>